<commit_message>
@ Add terminalID field alongside IMEI; unify 차량 상세 with 자원 관리
Resolves operator confusion where 자원 관리 showed Bike.imei (uploaded via
Excel) while 차량 상세 showed the device-installation deviceUid under the
"IMEI" label — two different values for the same vehicle.

- New Bike.terminalId (V39, varchar(64)), distinct from the 15-digit imei.
- BikeReadResponse exposes terminalId; BikeCreate/UpdateRequest now also
  accept imei + terminalId (previously imei was Excel-bulk-only).
- BikeBulkService parses/exports a 5th column (col4 = terminalID);
  vehicles-template.xlsx gains a "단말기 ID" column.
- 자원 관리 차량 table gains a 단말기 ID column.
- 차량 상세 now sources IMEI + 단말기 ID from the Bike record (identical to
  자원 관리) instead of the device deviceUid; the device-link input is kept
  but relabeled "단말기 연동 (deviceUid)" so it is no longer mistaken for IMEI.
  Edits to IMEI/terminalID persist to the Bike via updateVehicle.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/development/service-ops-api/src/main/resources/templates/excel/vehicles-template.xlsx
+++ b/development/service-ops-api/src/main/resources/templates/excel/vehicles-template.xlsx
@@ -498,13 +498,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D500"/>
+  <dimension ref="A1:E500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -538,6 +539,12 @@
 (선택, 15자리)</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>단말기 ID
+(terminalID)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -560,6 +567,11 @@
           <t>123456789012345</t>
         </is>
       </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>T0001</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -3573,7 +3585,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>